<commit_message>
build(track2-it2): the PDF and the xlsx re-rendered from the new sources
</commit_message>
<xml_diff>
--- a/submissions/track2/iteration-2/agharsallah_track2_methods_form.xlsx
+++ b/submissions/track2/iteration-2/agharsallah_track2_methods_form.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>From variant to mechanism to medicine in four documented stages, each a case-agnostic tool with a provenance manifest. (1) Hand-off: Track 1's confirmed compound-heterozygous BUB1B pair (a stop allele + a kinase-region missense, trans configuration confirmed by the challenge's answer key) was written into a structured 'mechanism card' (ressources/track2/mechanism.json): gene, protein, the two allele classes (never positions), loss-of-function reading, the spindle-assembly-checkpoint pathway, downstream consequences, the tumour context (rhabdomyosarcoma) from the clinical terms, and four repurposing directions with seed genes - D1 reinforce the checkpoint, D2 exploit aneuploidy stress, D3 stabilise the remaining BubR1 (hypomorph), D4 the child's tumour. Iteration 2 first rebuilt the genotype blind - a symptom-only target set with 396 matched decoy genes (step 1), alleles discovered from the raw reads without the vendor caller (step 2), alignment-free k-mer genotyping and copy number (step 3), a genome-wide likelihood-ratio ranking over 51,920 biallelic hypotheses (step 4), a public-knowledge route over 815 genes (step 5) and a rank fusion frozen by sha256 before it was compared (step 6): the same BUB1B pair came out first. Its measured facts (allele dosage, exon copy number, structural-variant absence, the missense's position in the protein, pathogenicity lanes, P(trans)) were appended as card revision v3, and step 8's mosaic-aneuploidy bound (fold-over allele-balance statistic, 80 % power at 2-3 % of cells, no autosome above its limit in the sequenced sample) as revision v4. (2) Search: the card's seeds were expanded through Reactome pathways to 277 targets; Open Targets, ChEMBL and DGIdb returned 3,859 drug-target rows and 359 market-approved drugs; openFDA confirmed US labels; ClinicalTrials.gov and PubMed answered trial and literature questions, all queries derived from the card. (3) Grading: every approved drug on every direction was placed on a five-rung evidence ladder pre-registered before the search (5 approved for a related indication with paediatric use; 4 trial in a related indication; 3 animal model of the mechanism; 2 cell model; 1 mechanism only - named, never submitted). Automated tests (approval, label and its Pediatric Use section, tumour-context trials, studies admitting children, PubMed co-mention counts) and curated tests (one PubMed paper per row, read by a person, 13 rows) are printed side by side; inherited class-level evidence is marked 'proxy'. Seven falsifiable claims (one per direction, one for the control, one for paediatric data, one that the measured aneuploid fraction moves no rung) were registered with predictions and refutation conditions before their tests; the last was tested by byte-identical table digests and caught a file-reading fault on the way. (4) Control: the same pipeline ran on two decoy cards - the child's clinical side kept, the gene swapped (NTRK3 by a seeded draw from Track 1's decoy set; XDH, an unrelated metabolic enzyme). A direction whose approved drugs overlap a decoy's at Jaccard &gt;= 0.10 is reported as non-specific; D4 did (0.25) and is argued only from curated mechanism results. Output: 11 drugs with a cited mechanism result (statins; niacin/nicotinamide; chloroquine; bortezomib, metformin, valproic acid, vorinostat, hydroxychloroquine, atorvastatin), 50 drugs already in rhabdomyosarcoma trials listed as such, and a 23-drug do-not table (spindle poisons, checkpoint inhibitors, standard of care).</t>
+          <t>From variant to mechanism to medicine in five documented stages, each a case-agnostic tool with a provenance manifest. (1) Hand-off: Track 1's confirmed compound-heterozygous BUB1B pair (a stop allele + a kinase-region missense, trans configuration confirmed by the challenge's answer key) was written into a structured 'mechanism card' (ressources/track2/mechanism.json): gene, protein, the two allele classes (never positions), loss-of-function reading, the spindle-assembly-checkpoint pathway, downstream consequences, the tumour context (rhabdomyosarcoma) from the clinical terms, and four repurposing directions with seed genes - D1 reinforce the checkpoint, D2 exploit aneuploidy stress, D3 stabilise the remaining BubR1 (hypomorph), D4 the child's tumour. Iteration 2 first rebuilt the genotype blind - a symptom-only target set with 396 matched decoy genes (step 1), alleles discovered from the raw reads without the vendor caller (step 2), alignment-free k-mer genotyping and copy number (step 3), a genome-wide likelihood-ratio ranking over 51,920 biallelic hypotheses (step 4), a public-knowledge route over 815 genes (step 5) and a rank fusion frozen by sha256 before it was compared (step 6): the same BUB1B pair came out first. Its measured facts (allele dosage, exon copy number, structural-variant absence, the missense's position in the protein, pathogenicity lanes, P(trans)) were appended as card revision v3, step 8's mosaic-aneuploidy bound (fold-over allele-balance statistic, 80 % power at 2-3 % of cells, no autosome above its limit in the sequenced sample) as revision v4, and step 8's second, independent instrument (k-mer dosage: one copy of X and one of Y recovered as a positive control, honest floor 1.6 % of cells) as revision v5. (2) Search: the card's seeds were expanded through Reactome pathways to 277 targets; Open Targets, ChEMBL and DGIdb returned 3,859 drug-target rows and 359 market-approved drugs; openFDA confirmed US labels; ClinicalTrials.gov and PubMed answered trial and literature questions, all queries derived from the card. (3) Grading: every approved drug on every direction was placed on a five-rung evidence ladder pre-registered before the search (5 approved for a related indication with paediatric use; 4 trial in a related indication; 3 animal model of the mechanism; 2 cell model; 1 mechanism only - named, never submitted). Automated tests (approval, label and its Pediatric Use section, tumour-context trials, studies admitting children, PubMed co-mention counts) and curated tests (one PubMed paper per row, read by a person, 13 rows) are printed side by side; inherited class-level evidence is marked 'proxy'. Every claim was registered with its prediction and its refutation condition before its test (one per direction, one for the control, one for paediatric data, one per card revision that the measured aneuploid fraction moves no rung, one for the transfer run); the card-revision tests were settled by byte-identical table digests, and the first of them caught a file-reading fault on the way. (4) Control: the same pipeline ran on two decoy cards - the child's clinical side kept, the gene swapped (NTRK3 by a seeded draw from Track 1's decoy set; XDH, an unrelated metabolic enzyme). A direction whose approved drugs overlap a decoy's at Jaccard &gt;= 0.10 is reported as non-specific; D4 did (0.25) and is argued only from curated mechanism results. This decoy card is the pipeline's negative control: it answers 'what does the same machinery return for a gene that is not the cause?', and a direction that cannot beat it is demoted rather than argued. (5) Transfer: the same pipeline then ran unchanged on a transfer card that swaps the whole case, not only the gene - TRIP13 / mosaic variegated aneuploidy syndrome 3, its own OMIM/MONDO identifiers, its own 19 HPO terms read out of the public HPO annotation file (phenotype.hpoa release 2026-09-02) rather than typed, its own nephroblastoma tumour context and standard of care, no alleles and no curated literature. No module was edited and no query was hand-written; it produced 28 targets, 277 approved drugs, a 370-row evidence ladder, a 53-row shortlist and a do-not table, with a provenance manifest per file and one comparison row per case in ressources/track2/transfer_comparison.tsv. Only the automated rungs (1, 4, 5) compare, because a transfer card has no curated evidence.tsv by construction. The transfer's pre-registered claim (H066) was written as a conjunction of five limbs and came back REFUTED (0.10), recorded as refuted rather than reworded: four limbs held, including every limb that tests portability (the run completed with no module edit; all 30 checkpoint-direction rows stayed at rung 1; no mechanism-direction row reached the 53-row shortlist; only the tumour-context direction rose above rung 1), and the fifth failed - the spindle-poison anti-direction populated no row of the transfer do-not table. Diagnosed cause, recorded with it: that flag is a regular expression over each drug's action-type and mechanism-of-action text, which arrives through pathway expansion, and Reactome matched no pathway for the transfer gene, so all 1,329 candidate rows stayed at seed role with only 261 carrying any mechanism text. The operational consequence is stated in the report: a new case's pathway coverage must be checked before its do-not table is trusted. Output: 11 drugs with a cited mechanism result (statins; niacin/nicotinamide; chloroquine; bortezomib, metformin, valproic acid, vorinostat, hydroxychloroquine, atorvastatin), 50 drugs already in rhabdomyosarcoma trials listed as such, and a 23-drug do-not table (spindle poisons, checkpoint inhibitors, standard of care).</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Loss of function, hypomorphic, of a confirmed compound heterozygote. One allele is a stop change in exon 17 of 23 (ClinVar pathogenic / likely pathogenic for MVA syndrome 1): no functional BubR1 from that copy. The other is a missense change in the last exon: absent from gnomAD, AlphaMissense likely-pathogenic (log-likelihood-ratio lane 4.33), CADD 24.5, sitting outside every InterPro domain-typed entry in a region AlphaFold models at pLDDT 91 - a weakened copy, not a dead one, consistent with every published MVA1 genotype (complete loss is embryonic-lethal). No gain-of-function or dominant-negative activity is reported for BUB1B. Trans configuration: confirmed by the oracle's full match at rank 1 (population phasing was undetermined; read-backed phase blocks did not reach the gene). Dosage: both alleles at one-copy multiplicity in the raw reads by an alignment-free k-mer method; every exon at two copies; no structural variant in the gene. Pathway: the spindle assembly checkpoint - BubR1 is a core component of the mitotic checkpoint complex that inhibits APC/C-CDC20 and recruits PP2A-B56 to kinetochores; less BubR1 gives a leaky checkpoint (Suijkerbuijk 2010 measured strongly reduced BubR1 and a weakened checkpoint in MVA cells). Downstream: premature anaphase and chromosome missegregation; mosaic variegated aneuploidy; proteotoxic and metabolic stress in aneuploid cells; cancer predisposition (rhabdomyosarcoma - the child's presenting tumour - Wilms tumour, leukaemia); growth restriction and nephrocalcinosis, which are the delivered clinical terms. Aneuploid fraction: measured in iteration 2's step 8 - a fold-over B-allele-deviation statistic with 80 % power at 2 % (chr1-6) and 3 % (chr7-22) of cells finds no autosome above its own detection limit in the sequenced sample (the statistic used earlier, the mean B-allele fraction per megabase, had no power at any fraction tested); X and Y are unreadable by allele balance in a male, sub-arm events were not testable, and the sequenced tissue is not named by the delivery, so this is a statement about the sample and not the diagnosis. Consequence for the drug argument: direction D2 (aneuploidy-selective stress) is argued from published aneuploid-cell biology only and ranked below D3 and D4. Open: whether the missense copy is unstable or catalytically inactive - so D3 is argued as raising BubR1 abundance, not as refolding it.</t>
+          <t>Loss of function, hypomorphic, of a confirmed compound heterozygote. One allele is a stop change in exon 17 of 23 (ClinVar pathogenic / likely pathogenic for MVA syndrome 1): no functional BubR1 from that copy. The other is a missense change in the last exon: absent from gnomAD, AlphaMissense likely-pathogenic (log-likelihood-ratio lane 4.33), CADD 24.5, sitting outside every InterPro domain-typed entry in a region AlphaFold models at pLDDT 91 - a weakened copy, not a dead one, consistent with every published MVA1 genotype (complete loss is embryonic-lethal). No gain-of-function or dominant-negative activity is reported for BUB1B. Trans configuration: confirmed by the oracle's full match at rank 1 (population phasing was undetermined; read-backed phase blocks did not reach the gene). Dosage: both alleles at one-copy multiplicity in the raw reads by an alignment-free k-mer method; every exon at two copies; no structural variant in the gene. Pathway: the spindle assembly checkpoint - BubR1 is a core component of the mitotic checkpoint complex that inhibits APC/C-CDC20 and recruits PP2A-B56 to kinetochores; less BubR1 gives a leaky checkpoint (Suijkerbuijk 2010 measured strongly reduced BubR1 and a weakened checkpoint in MVA cells). Downstream: premature anaphase and chromosome missegregation; mosaic variegated aneuploidy; proteotoxic and metabolic stress in aneuploid cells; cancer predisposition (rhabdomyosarcoma - the child's presenting tumour - Wilms tumour, leukaemia); growth restriction and nephrocalcinosis, which are the delivered clinical terms. Aneuploid fraction: measured in iteration 2's step 8 by two instruments that share nothing past the raw reads. Instrument 1, allele balance: a fold-over B-allele-deviation statistic with 80 % power at 2 % (chr1-6) and 3 % (chr7-22) of cells finds no autosome above its own detection limit in the sequenced sample (the statistic used earlier, the mean B-allele fraction per megabase, had no power at any fraction tested); it cannot read X or Y in a male. Instrument 2, k-mer dosage (reference-unique 31-mers over 32 of 272 flowcell shards): recovers one copy of X at 0.4873 and one of Y at 0.5083 against 0.5 expected - the positive control allele balance cannot supply - and puts no autosome beyond its composition-corrected null (chromosome-GC regressor, Pearson 0.904, 81.7 % of the between-chromosome spread explained, residual spread 0.802 %); the one chromosome that looked suspicious under a bootstrap interval (chr21, 2.33 sigma, Bonferroni p 0.43) dissolved under tail trimming, a probe half-split and a depth check that read the excess as mismapping pileups. Honest floor: 1.6 % of cells, twice the residual spread. Still outside both routes: events smaller than a chromosome arm, and copy-neutral loss of heterozygosity, which moves no sequence for the dosage route to see; and the sequenced tissue is not named by the delivery, so this is a statement about the sample and not the diagnosis. Consequence for the drug argument: direction D2 (aneuploidy-selective stress) is argued from published aneuploid-cell biology only and ranked below D3 and D4. Open: whether the missense copy is unstable or catalytically inactive - so D3 is argued as raising BubR1 abundance, not as refolding it.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Roughly five working days across two people-equivalents for Track 2 itself (the card and data layer on 2026-09-05/06; the claims, ladder, decoy control, curation, figures, dashboard and report on 2026-09-18; the card revision from step 8 and this report on 2026-09-19), on top of the fortnight of iteration-2 genotype work (steps 1-6 and 8) the mechanism facts come from. Compute for Track 2: two laptop runs of about ten minutes against public APIs; no cloud.</t>
+          <t>Roughly five working days across two people-equivalents for Track 2 itself (the card and data layer on 2026-09-05/06; the claims, ladder, decoy control, curation, figures, dashboard and report on 2026-09-18; the card revision from step 8 and this report on 2026-09-19), on top of the fortnight of iteration-2 genotype work (steps 1-6 and 8) the mechanism facts come from. Compute for Track 2: two laptop runs of about ten minutes against public APIs; no cloud, no paid data source, so the marginal money cost of a run is zero. Measured cost of adding a case the pipeline had never seen (the TRIP13 transfer run, cold cache): 2,077 live requests and 1,693.7 s of wall clock end to end on the same laptop, of which about 706 s is the enforced 0.34 s politeness interval between live calls; re-deriving the same tables from the warm cache afterwards took 9.0 s. The real case's own 85 live requests are not comparable, because they were measured against a cache 1,965 replies deep.</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Question. Given a confirmed compound-heterozygous loss of BUB1B (a stop allele and a hypomorphic kinase-region missense) in a child with mosaic variegated aneuploidy and rhabdomyosarcoma, which market-approved drugs act on the mechanism, and how strong is the evidence for each? Method. Iteration 2 first rebuilt the genotype blind from the raw reads and the eight clinical terms - symptom-only target set with matched decoys, alleles from the reads without the vendor caller, alignment-free genotyping and copy number, a genome-wide likelihood ranking, a knowledge route, and a rank fusion frozen by digest before comparison - and found the same pair first. A structured mechanism card carries the confirmed pair and nine measured facts, the ninth being step 8's mosaic-aneuploidy bound (80 % power at 2-3 % of cells; no autosome above its limit in the sequenced sample). The card drives every query: Reactome expands its seeds to 277 targets; Open Targets, ChEMBL and DGIdb return 359 approved drugs; openFDA, ClinicalTrials.gov and PubMed answer label, trial and literature questions per drug. Every drug on every direction is placed on a five-rung evidence ladder pre-registered before the search, automated tests beside 13 person-curated PubMed rows, inherited class evidence flagged as proxy. Seven claims were registered with refutation conditions before their tests. The pipeline ran unchanged on two decoy cards (same child, gene swapped) as a specificity control. Results. D1 (reinforce the checkpoint) has no approved drug and became the do-not table. D3 (raise BubR1): NAD+ repletion raised BubR1 in BubR1-hypomorphic mice, inherited by niacin and nicotinamide (rung 3); HDAC inhibitors act on BubR1's acetylation switch at class level. D4 (the tumour): lovastatin itself slowed rhabdomyosarcoma cells and a completed paediatric phase-1 trial gave simvastatin in relapsed solid tumours including rhabdomyosarcoma. D2 (aneuploidy stress): chloroquine has a molecule-level cell result, but the direction is argued from the literature only and ranked last, because the sequenced sample shows no aneuploid population for such a drug to act on. Eleven drugs carry a cited mechanism result; fifty more reach the top rung only because they are already in rhabdomyosarcoma trials and are listed, not claimed. The decoy control showed D4's automated stage non-specific (Jaccard 0.25) and D1-D3 specific, and exposed a grading flaw corrected before any verdict; a second pre-registered test showed the measured aneuploid fraction moved no rung. The do-not table names 13 spindle poisons - including standard rhabdomyosarcoma chemotherapy - as a caution for the treating team, because they rely on the very checkpoint that is weakened. Strengths. Pre-registration; a decoy control for a repurposing pipeline; automated and curated evidence never merged; complete lineage; case-agnostic tooling; no patient data in any Track 2 artefact. Limitations. Curated rungs are one reader's; rung 3 is one mouse paper; the aneuploid fraction is measured in a sample whose tissue is unnamed, for whole chromosomes and arms only; the missense's unstable-versus-inactive status is open; DrugBank was not queried; a paediatric pointer is not safety data. These are hypotheses for follow-up, not evidence that any medicine works.</t>
+          <t>Question. Given a confirmed compound-heterozygous loss of BUB1B (a stop allele and a hypomorphic kinase-region missense) in a child with mosaic variegated aneuploidy and rhabdomyosarcoma, which market-approved drugs act on the mechanism, and how strong is the evidence for each? Method. We first rebuilt the genotype blind from the raw reads and the eight clinical terms - symptom-only target set with matched decoys, alleles from the reads without the vendor caller, alignment-free genotyping, a genome-wide likelihood ranking, a knowledge route, and a rank fusion frozen by digest before comparison - and found the same pair first. A structured mechanism card carries the confirmed pair and nine measured facts. The ninth, step 8's mosaic-aneuploidy bound, is now measured by two instruments sharing nothing past the raw reads: allele balance (80 % power at 2-3 % of cells; no autosome above its limit) and k-mer dosage, recovering one copy each of X and Y as a positive control and setting a 1.6 % floor. The card drives every query: Reactome expands its seeds to 277 targets; Open Targets, ChEMBL and DGIdb return 359 approved drugs; openFDA, ClinicalTrials.gov and PubMed answer label, trial and literature questions per drug. Every drug on every direction sits on a five-rung ladder pre-registered before the search, automated tests beside 13 person-curated PubMed rows, inherited class evidence flagged as proxy. Claims were registered with predictions and refutation conditions before their tests. Controls: two decoy cards (same child, gene swapped) and a transfer card swapping the whole case (TRIP13 / MVA syndrome 3, nephroblastoma, its own phenotype terms read from public annotation), both run unchanged. Results. D1 (reinforce the checkpoint) has no approved drug and became the do-not table. D3 (raise BubR1): NAD+ repletion raised BubR1 in BubR1-hypomorphic mice, inherited by niacin and nicotinamide (rung 3); HDAC inhibitors act on BubR1's acetylation switch at class level. D4 (the tumour): lovastatin itself slowed rhabdomyosarcoma cells, and a completed paediatric phase-1 trial gave simvastatin in relapsed solid tumours. D2 (aneuploidy stress): chloroquine has a molecule-level cell result, but the direction is literature-only and ranked last: the sequenced sample shows no aneuploid population for such a drug to act on. Eleven drugs carry a cited mechanism result; fifty more reach the top rung only as tumour-trial context, listed not claimed; 23 sit in the do-not table, among them 13 spindle poisons relying on the very checkpoint that is broken. The decoy control showed D4's automated stage non-specific (Jaccard 0.25) and exposed a grading flaw, corrected before any verdict; two pre-registered digest tests showed neither card revision moved a rung; the transfer case produced a complete output with no code change, D1 again empty. Limitations. Curated rungs are one reader's; rung 3 is one mouse paper; the aneuploidy bound covers whole chromosomes and arms in a sample whose tissue is unnamed; the transfer case has no curated evidence, so only automated rungs compare; DrugBank was not queried. Hypotheses for follow-up, not evidence that any medicine works.</t>
         </is>
       </c>
     </row>

</xml_diff>